<commit_message>
Add concave/convex/linear notes and MU utility graphs to guide
- NEGATIVE: concave utility, MU decreasing, u'' < 0 (risk averse)
- POSITIVE: convex utility, MU increasing, u'' > 0 (risk loving)
- NEUTRAL: linear utility, flat MU, u'' = 0 (risk neutral)
- Graphs for sqrt(x), x, and x^2 with matching MU curves

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Marginal_Utility_Guide.xlsx
+++ b/Marginal_Utility_Guide.xlsx
@@ -334,6 +334,81 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>383</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>446</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>510</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -709,79 +784,79 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Extra satisfaction from exactly one more unit. MU = change in TU.</t>
+          <t>Extra satisfaction from exactly one more unit. MU = u'(x).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>First derivative</t>
+          <t>Second derivative</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>MU = u'(I). Answers: how much does the next unit add?</t>
+          <t>Measures whether MU is increasing, decreasing, or flat.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Second derivative</t>
+          <t>MU increasing example</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Rate of change of MU. Is MU rising, falling, or flat?</t>
+          <t>MU at 1 = 10, MU at 2 = 20 -&gt; MU rising -&gt; u'' &gt; 0 -&gt; risk-loving</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>MU increasing</t>
+          <t>NEGATIVE u''</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Example: MU at unit 1 = 10, MU at unit 2 = 20 -&gt; MU rising -&gt; u'' &gt; 0 -&gt; risk-loving</t>
+          <t>Concave utility. MU going down. Second derivative negative because MU is decreasing. Risk averse.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>MU decreasing</t>
+          <t>POSITIVE u''</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Each extra unit adds less -&gt; u'' &lt; 0 -&gt; risk-averse (most common on exam)</t>
+          <t>Convex utility. MU going up, faster every unit. Risk loving.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>MU constant</t>
+          <t>NEUTRAL u'' = 0</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Each extra unit adds the same -&gt; u'' = 0 -&gt; risk-neutral</t>
+          <t>Linear utility. Flat MU line. Second derivative is 0. Risk neutral.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Exam shortcut</t>
+          <t>Graphs in PDF</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>u'' &lt; 0: risk averse | u'' = 0: risk neutral | u'' &gt; 0: risk loving</t>
+          <t>sqrt(x) concave + decreasing MU | x linear + flat MU | x^2 convex + increasing MU</t>
         </is>
       </c>
     </row>

</xml_diff>